<commit_message>
chore: updated the repos and removed the xslx files
</commit_message>
<xml_diff>
--- a/saved/giardia/Giardia_bot_activity_09_02_2025.xlsx
+++ b/saved/giardia/Giardia_bot_activity_09_02_2025.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -705,126 +705,6 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>CAS10988009ME01</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Reject Notification</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Specimen source doesn't match lab report: Needs manual review.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>CAS10988008ME01</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Approve Notification</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>CAS10988010ME01</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Approve Notification</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>CAS10988011ME01</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Reject Notification</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Specimen source doesn't match lab report: Needs manual review.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>CAS10988012ME01</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Approve Notification</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>CAS10991001ME01</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Approve Notification</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Approved</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>